<commit_message>
Fix : ne pas définir password="" sur la protection
openpyxl interprète password="" comme une chaîne à hasher (résultat : 'CE4B'),
ce qui rend la feuille inéditable même pour les cellules déverrouillées.

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/TRAME_260512_NOTES_BAC_BLANC_N°2_v2.xlsx
+++ b/TRAME_260512_NOTES_BAC_BLANC_N°2_v2.xlsx
@@ -1489,7 +1489,7 @@
       </c>
     </row>
   </sheetData>
-  <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="1" scenarios="0" formatColumns="1" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="1" sort="1" password="CE4B"/>
+  <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="1" scenarios="0" formatColumns="1" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="1" sort="1"/>
   <mergeCells count="1">
     <mergeCell ref="A1:F1"/>
   </mergeCells>
@@ -13238,7 +13238,7 @@
       </c>
     </row>
   </sheetData>
-  <sheetProtection selectLockedCells="1" selectUnlockedCells="1" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="1" scenarios="0" formatColumns="0" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="0" formatRows="0" sort="1" password="CE4B"/>
+  <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="1" scenarios="0" formatColumns="0" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="0" formatRows="0" sort="1"/>
   <mergeCells count="2">
     <mergeCell ref="A2:CR2"/>
     <mergeCell ref="A1:CR1"/>

</xml_diff>